<commit_message>
sc-infra-categories: cyrillic labels + updated sc.xlsx template
The five sc_infra_event_categories were seeded with latin-script labels
in 000066. Those labels show up verbatim as the section headers in the
SC daily Excel report, which is read in Uzbek-Cyrillic.

Migration 000087 rewrites the labels in place (matched by slug) and the
template was nudged to match the new wider Cyrillic strings. slug and
display_name are untouched — display_name is the admin-UI Russian label
and was already correct.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internal/lib/service/excel/templates/sc.xlsx
+++ b/internal/lib/service/excel/templates/sc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ЭтаКнига" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\go\srmt-prime\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\go\srmt-prime\internal\lib\service\excel\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8789F035-7003-4380-808F-BE76AFF296C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE9E8C76-7F3A-448F-AFBD-53806D317CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38535" yWindow="-5460" windowWidth="38670" windowHeight="21150" xr2:uid="{2CF4B48C-F2A4-4814-9FBC-8CF197464069}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CF4B48C-F2A4-4814-9FBC-8CF197464069}"/>
   </bookViews>
   <sheets>
     <sheet name="Ўчишлар В1 ойлик" sheetId="1" r:id="rId1"/>
@@ -65,9 +65,6 @@
     <t>Юз берган сана ва вақти</t>
   </si>
   <si>
-    <t>Тиклан-ган сана ва вақти</t>
-  </si>
-  <si>
     <t>Аварияни келиб чиқиш сабаблари</t>
   </si>
   <si>
@@ -225,9 +222,6 @@
 тезкор навбатчиси</t>
   </si>
   <si>
-    <t>Давомий-лиги</t>
-  </si>
-  <si>
     <t>Аниқланган носозлик</t>
   </si>
   <si>
@@ -235,6 +229,12 @@
   </si>
   <si>
     <t>infra</t>
+  </si>
+  <si>
+    <t>Тикланган сана ва вақти</t>
+  </si>
+  <si>
+    <t>Давомийлиги</t>
   </si>
 </sst>
 </file>
@@ -721,7 +721,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -953,6 +953,75 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -962,230 +1031,158 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1525,23 +1522,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:68" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="137" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="138"/>
-      <c r="O1" s="138"/>
+      <c r="A1" s="111" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="112"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="112"/>
+      <c r="L1" s="112"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="112"/>
+      <c r="O1" s="112"/>
     </row>
     <row r="2" spans="1:68" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="38"/>
@@ -1561,23 +1558,23 @@
       <c r="O2" s="39"/>
     </row>
     <row r="3" spans="1:68" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="95" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="90"/>
-      <c r="M3" s="90"/>
-      <c r="N3" s="90"/>
-      <c r="O3" s="91"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="96"/>
+      <c r="J3" s="96"/>
+      <c r="K3" s="96"/>
+      <c r="L3" s="96"/>
+      <c r="M3" s="96"/>
+      <c r="N3" s="96"/>
+      <c r="O3" s="97"/>
       <c r="P3" s="60"/>
     </row>
     <row r="4" spans="1:68" ht="27" customHeight="1" x14ac:dyDescent="0.25">
@@ -1587,98 +1584,98 @@
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="139" t="s">
+      <c r="C4" s="90" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="139"/>
-      <c r="E4" s="139"/>
-      <c r="F4" s="139" t="s">
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="139"/>
-      <c r="H4" s="139"/>
-      <c r="I4" s="139"/>
-      <c r="J4" s="139"/>
-      <c r="K4" s="139"/>
-      <c r="L4" s="139"/>
-      <c r="M4" s="139"/>
-      <c r="N4" s="139"/>
-      <c r="O4" s="139"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="90"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="90"/>
+      <c r="N4" s="90"/>
+      <c r="O4" s="90"/>
       <c r="P4" s="60" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:68" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="42"/>
-      <c r="C5" s="82"/>
-      <c r="D5" s="101"/>
-      <c r="E5" s="101"/>
-      <c r="F5" s="144"/>
-      <c r="G5" s="101"/>
-      <c r="H5" s="101"/>
-      <c r="I5" s="101"/>
-      <c r="J5" s="101"/>
-      <c r="K5" s="101"/>
-      <c r="L5" s="101"/>
-      <c r="M5" s="101"/>
-      <c r="N5" s="101"/>
-      <c r="O5" s="102"/>
+      <c r="C5" s="105"/>
+      <c r="D5" s="117"/>
+      <c r="E5" s="117"/>
+      <c r="F5" s="118"/>
+      <c r="G5" s="117"/>
+      <c r="H5" s="117"/>
+      <c r="I5" s="117"/>
+      <c r="J5" s="117"/>
+      <c r="K5" s="117"/>
+      <c r="L5" s="117"/>
+      <c r="M5" s="117"/>
+      <c r="N5" s="117"/>
+      <c r="O5" s="119"/>
       <c r="P5" s="60"/>
     </row>
     <row r="6" spans="1:68" ht="16.8" x14ac:dyDescent="0.25">
       <c r="A6" s="54"/>
       <c r="B6" s="55"/>
-      <c r="C6" s="140"/>
-      <c r="D6" s="141"/>
-      <c r="E6" s="141"/>
-      <c r="F6" s="142"/>
-      <c r="G6" s="141"/>
-      <c r="H6" s="141"/>
-      <c r="I6" s="141"/>
-      <c r="J6" s="141"/>
-      <c r="K6" s="141"/>
-      <c r="L6" s="141"/>
-      <c r="M6" s="141"/>
-      <c r="N6" s="141"/>
-      <c r="O6" s="141"/>
+      <c r="C6" s="113"/>
+      <c r="D6" s="114"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="115"/>
+      <c r="G6" s="114"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="114"/>
+      <c r="J6" s="114"/>
+      <c r="K6" s="114"/>
+      <c r="L6" s="114"/>
+      <c r="M6" s="114"/>
+      <c r="N6" s="114"/>
+      <c r="O6" s="114"/>
     </row>
     <row r="7" spans="1:68" ht="0.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="143"/>
-      <c r="B7" s="143"/>
-      <c r="C7" s="143"/>
-      <c r="D7" s="143"/>
-      <c r="E7" s="143"/>
-      <c r="F7" s="143"/>
-      <c r="G7" s="143"/>
-      <c r="H7" s="143"/>
-      <c r="I7" s="143"/>
-      <c r="J7" s="143"/>
-      <c r="K7" s="143"/>
-      <c r="L7" s="143"/>
-      <c r="M7" s="143"/>
-      <c r="N7" s="143"/>
-      <c r="O7" s="143"/>
+      <c r="A7" s="116"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
+      <c r="H7" s="116"/>
+      <c r="I7" s="116"/>
+      <c r="J7" s="116"/>
+      <c r="K7" s="116"/>
+      <c r="L7" s="116"/>
+      <c r="M7" s="116"/>
+      <c r="N7" s="116"/>
+      <c r="O7" s="116"/>
       <c r="P7" s="60"/>
     </row>
     <row r="8" spans="1:68" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="89" t="s">
+      <c r="A8" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="90"/>
-      <c r="C8" s="90"/>
-      <c r="D8" s="90"/>
-      <c r="E8" s="90"/>
-      <c r="F8" s="90"/>
-      <c r="G8" s="90"/>
-      <c r="H8" s="90"/>
-      <c r="I8" s="90"/>
-      <c r="J8" s="90"/>
-      <c r="K8" s="90"/>
-      <c r="L8" s="90"/>
-      <c r="M8" s="90"/>
-      <c r="N8" s="90"/>
-      <c r="O8" s="91"/>
+      <c r="B8" s="96"/>
+      <c r="C8" s="96"/>
+      <c r="D8" s="96"/>
+      <c r="E8" s="96"/>
+      <c r="F8" s="96"/>
+      <c r="G8" s="96"/>
+      <c r="H8" s="96"/>
+      <c r="I8" s="96"/>
+      <c r="J8" s="96"/>
+      <c r="K8" s="96"/>
+      <c r="L8" s="96"/>
+      <c r="M8" s="96"/>
+      <c r="N8" s="96"/>
+      <c r="O8" s="97"/>
       <c r="P8" s="60"/>
     </row>
     <row r="9" spans="1:68" s="3" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1692,29 +1689,29 @@
         <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="108" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="134" t="s">
+      <c r="F9" s="109"/>
+      <c r="G9" s="109"/>
+      <c r="H9" s="109"/>
+      <c r="I9" s="110"/>
+      <c r="J9" s="108" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="135"/>
-      <c r="G9" s="135"/>
-      <c r="H9" s="135"/>
-      <c r="I9" s="136"/>
-      <c r="J9" s="134" t="s">
+      <c r="K9" s="109"/>
+      <c r="L9" s="109"/>
+      <c r="M9" s="110"/>
+      <c r="N9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K9" s="135"/>
-      <c r="L9" s="135"/>
-      <c r="M9" s="136"/>
-      <c r="N9" s="1" t="s">
+      <c r="O9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O9" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="P9" s="60" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
@@ -1776,15 +1773,15 @@
       <c r="B10" s="5"/>
       <c r="C10" s="41"/>
       <c r="D10" s="41"/>
-      <c r="E10" s="82"/>
-      <c r="F10" s="83"/>
-      <c r="G10" s="83"/>
-      <c r="H10" s="83"/>
-      <c r="I10" s="84"/>
-      <c r="J10" s="82"/>
-      <c r="K10" s="83"/>
-      <c r="L10" s="83"/>
-      <c r="M10" s="83"/>
+      <c r="E10" s="105"/>
+      <c r="F10" s="106"/>
+      <c r="G10" s="106"/>
+      <c r="H10" s="106"/>
+      <c r="I10" s="107"/>
+      <c r="J10" s="105"/>
+      <c r="K10" s="106"/>
+      <c r="L10" s="106"/>
+      <c r="M10" s="106"/>
       <c r="N10" s="8"/>
       <c r="O10" s="58"/>
       <c r="P10" s="52"/>
@@ -1794,17 +1791,17 @@
       <c r="B11" s="61"/>
       <c r="C11" s="61"/>
       <c r="D11" s="62"/>
-      <c r="E11" s="85" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="86"/>
-      <c r="G11" s="86"/>
-      <c r="H11" s="86"/>
-      <c r="I11" s="86"/>
-      <c r="J11" s="86"/>
-      <c r="K11" s="86"/>
-      <c r="L11" s="86"/>
-      <c r="M11" s="87"/>
+      <c r="E11" s="99" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="100"/>
+      <c r="G11" s="100"/>
+      <c r="H11" s="100"/>
+      <c r="I11" s="100"/>
+      <c r="J11" s="100"/>
+      <c r="K11" s="100"/>
+      <c r="L11" s="100"/>
+      <c r="M11" s="101"/>
       <c r="N11" s="7">
         <v>0</v>
       </c>
@@ -1814,43 +1811,43 @@
       <c r="P11" s="60"/>
     </row>
     <row r="12" spans="1:68" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A12" s="88"/>
-      <c r="B12" s="88"/>
-      <c r="C12" s="88"/>
-      <c r="D12" s="88"/>
-      <c r="E12" s="88"/>
-      <c r="F12" s="88"/>
-      <c r="G12" s="88"/>
-      <c r="H12" s="88"/>
-      <c r="I12" s="88"/>
-      <c r="J12" s="88"/>
-      <c r="K12" s="88"/>
-      <c r="L12" s="88"/>
-      <c r="M12" s="88"/>
-      <c r="N12" s="88"/>
-      <c r="O12" s="88"/>
+      <c r="A12" s="158"/>
+      <c r="B12" s="158"/>
+      <c r="C12" s="158"/>
+      <c r="D12" s="158"/>
+      <c r="E12" s="158"/>
+      <c r="F12" s="158"/>
+      <c r="G12" s="158"/>
+      <c r="H12" s="158"/>
+      <c r="I12" s="158"/>
+      <c r="J12" s="158"/>
+      <c r="K12" s="158"/>
+      <c r="L12" s="158"/>
+      <c r="M12" s="158"/>
+      <c r="N12" s="158"/>
+      <c r="O12" s="158"/>
       <c r="P12" s="60"/>
     </row>
     <row r="13" spans="1:68" s="2" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="89" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="90"/>
-      <c r="H13" s="90"/>
-      <c r="I13" s="90"/>
-      <c r="J13" s="90"/>
-      <c r="K13" s="90"/>
-      <c r="L13" s="90"/>
-      <c r="M13" s="90"/>
-      <c r="N13" s="90"/>
-      <c r="O13" s="91"/>
+      <c r="A13" s="95" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="96"/>
+      <c r="C13" s="96"/>
+      <c r="D13" s="96"/>
+      <c r="E13" s="96"/>
+      <c r="F13" s="96"/>
+      <c r="G13" s="96"/>
+      <c r="H13" s="96"/>
+      <c r="I13" s="96"/>
+      <c r="J13" s="96"/>
+      <c r="K13" s="96"/>
+      <c r="L13" s="96"/>
+      <c r="M13" s="96"/>
+      <c r="N13" s="96"/>
+      <c r="O13" s="97"/>
       <c r="P13" s="60" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:68" s="2" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -1860,15 +1857,15 @@
       <c r="B14" s="5"/>
       <c r="C14" s="50"/>
       <c r="D14" s="50"/>
-      <c r="E14" s="82"/>
-      <c r="F14" s="83"/>
-      <c r="G14" s="83"/>
-      <c r="H14" s="83"/>
-      <c r="I14" s="84"/>
-      <c r="J14" s="82"/>
-      <c r="K14" s="92"/>
-      <c r="L14" s="92"/>
-      <c r="M14" s="92"/>
+      <c r="E14" s="105"/>
+      <c r="F14" s="106"/>
+      <c r="G14" s="106"/>
+      <c r="H14" s="106"/>
+      <c r="I14" s="107"/>
+      <c r="J14" s="105"/>
+      <c r="K14" s="142"/>
+      <c r="L14" s="142"/>
+      <c r="M14" s="142"/>
       <c r="N14" s="8"/>
       <c r="O14" s="8"/>
       <c r="P14" s="63"/>
@@ -1878,17 +1875,17 @@
       <c r="B15" s="5"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
-      <c r="E15" s="85" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="86"/>
-      <c r="G15" s="86"/>
-      <c r="H15" s="86"/>
-      <c r="I15" s="86"/>
-      <c r="J15" s="86"/>
-      <c r="K15" s="86"/>
-      <c r="L15" s="86"/>
-      <c r="M15" s="87"/>
+      <c r="E15" s="99" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="100"/>
+      <c r="G15" s="100"/>
+      <c r="H15" s="100"/>
+      <c r="I15" s="100"/>
+      <c r="J15" s="100"/>
+      <c r="K15" s="100"/>
+      <c r="L15" s="100"/>
+      <c r="M15" s="101"/>
       <c r="N15" s="7">
         <v>0</v>
       </c>
@@ -1916,25 +1913,25 @@
       <c r="P16" s="60"/>
     </row>
     <row r="17" spans="1:16" s="2" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="89" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="90"/>
-      <c r="C17" s="90"/>
-      <c r="D17" s="90"/>
-      <c r="E17" s="90"/>
-      <c r="F17" s="90"/>
-      <c r="G17" s="90"/>
-      <c r="H17" s="90"/>
-      <c r="I17" s="90"/>
-      <c r="J17" s="90"/>
-      <c r="K17" s="90"/>
-      <c r="L17" s="90"/>
-      <c r="M17" s="90"/>
-      <c r="N17" s="90"/>
-      <c r="O17" s="91"/>
+      <c r="A17" s="95" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="96"/>
+      <c r="C17" s="96"/>
+      <c r="D17" s="96"/>
+      <c r="E17" s="96"/>
+      <c r="F17" s="96"/>
+      <c r="G17" s="96"/>
+      <c r="H17" s="96"/>
+      <c r="I17" s="96"/>
+      <c r="J17" s="96"/>
+      <c r="K17" s="96"/>
+      <c r="L17" s="96"/>
+      <c r="M17" s="96"/>
+      <c r="N17" s="96"/>
+      <c r="O17" s="97"/>
       <c r="P17" s="60" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:16" s="2" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -1944,11 +1941,11 @@
       <c r="B18" s="5"/>
       <c r="C18" s="41"/>
       <c r="D18" s="50"/>
-      <c r="E18" s="82"/>
-      <c r="F18" s="83"/>
-      <c r="G18" s="83"/>
-      <c r="H18" s="83"/>
-      <c r="I18" s="84"/>
+      <c r="E18" s="105"/>
+      <c r="F18" s="106"/>
+      <c r="G18" s="106"/>
+      <c r="H18" s="106"/>
+      <c r="I18" s="107"/>
       <c r="J18" s="51"/>
       <c r="K18" s="51"/>
       <c r="L18" s="51"/>
@@ -1962,17 +1959,17 @@
       <c r="B19" s="5"/>
       <c r="C19" s="41"/>
       <c r="D19" s="41"/>
-      <c r="E19" s="85" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" s="86"/>
-      <c r="G19" s="86"/>
-      <c r="H19" s="86"/>
-      <c r="I19" s="86"/>
-      <c r="J19" s="86"/>
-      <c r="K19" s="86"/>
-      <c r="L19" s="86"/>
-      <c r="M19" s="87"/>
+      <c r="E19" s="99" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="100"/>
+      <c r="G19" s="100"/>
+      <c r="H19" s="100"/>
+      <c r="I19" s="100"/>
+      <c r="J19" s="100"/>
+      <c r="K19" s="100"/>
+      <c r="L19" s="100"/>
+      <c r="M19" s="101"/>
       <c r="N19" s="7">
         <v>0</v>
       </c>
@@ -1986,17 +1983,17 @@
       <c r="B20" s="15"/>
       <c r="C20" s="43"/>
       <c r="D20" s="6"/>
-      <c r="E20" s="146" t="s">
-        <v>16</v>
-      </c>
-      <c r="F20" s="147"/>
-      <c r="G20" s="147"/>
-      <c r="H20" s="147"/>
-      <c r="I20" s="147"/>
-      <c r="J20" s="147"/>
-      <c r="K20" s="147"/>
-      <c r="L20" s="147"/>
-      <c r="M20" s="148"/>
+      <c r="E20" s="102" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="103"/>
+      <c r="G20" s="103"/>
+      <c r="H20" s="103"/>
+      <c r="I20" s="103"/>
+      <c r="J20" s="103"/>
+      <c r="K20" s="103"/>
+      <c r="L20" s="103"/>
+      <c r="M20" s="104"/>
       <c r="N20" s="7">
         <f>+N19+N15+N11</f>
         <v>0</v>
@@ -2008,109 +2005,109 @@
       <c r="P20" s="60"/>
     </row>
     <row r="21" spans="1:16" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A21" s="145"/>
-      <c r="B21" s="145"/>
-      <c r="C21" s="145"/>
-      <c r="D21" s="145"/>
-      <c r="E21" s="145"/>
-      <c r="F21" s="145"/>
-      <c r="G21" s="145"/>
-      <c r="H21" s="145"/>
-      <c r="I21" s="145"/>
-      <c r="J21" s="145"/>
-      <c r="K21" s="145"/>
-      <c r="L21" s="145"/>
-      <c r="M21" s="145"/>
-      <c r="N21" s="145"/>
-      <c r="O21" s="145"/>
+      <c r="A21" s="98"/>
+      <c r="B21" s="98"/>
+      <c r="C21" s="98"/>
+      <c r="D21" s="98"/>
+      <c r="E21" s="98"/>
+      <c r="F21" s="98"/>
+      <c r="G21" s="98"/>
+      <c r="H21" s="98"/>
+      <c r="I21" s="98"/>
+      <c r="J21" s="98"/>
+      <c r="K21" s="98"/>
+      <c r="L21" s="98"/>
+      <c r="M21" s="98"/>
+      <c r="N21" s="98"/>
+      <c r="O21" s="98"/>
       <c r="P21" s="60"/>
     </row>
     <row r="22" spans="1:16" s="2" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="89" t="s">
+      <c r="A22" s="95" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="96"/>
+      <c r="C22" s="96"/>
+      <c r="D22" s="96"/>
+      <c r="E22" s="96"/>
+      <c r="F22" s="96"/>
+      <c r="G22" s="96"/>
+      <c r="H22" s="96"/>
+      <c r="I22" s="96"/>
+      <c r="J22" s="96"/>
+      <c r="K22" s="96"/>
+      <c r="L22" s="96"/>
+      <c r="M22" s="96"/>
+      <c r="N22" s="96"/>
+      <c r="O22" s="97"/>
+      <c r="P22" s="64"/>
+    </row>
+    <row r="23" spans="1:16" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="122" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="90"/>
-      <c r="C22" s="90"/>
-      <c r="D22" s="90"/>
-      <c r="E22" s="90"/>
-      <c r="F22" s="90"/>
-      <c r="G22" s="90"/>
-      <c r="H22" s="90"/>
-      <c r="I22" s="90"/>
-      <c r="J22" s="90"/>
-      <c r="K22" s="90"/>
-      <c r="L22" s="90"/>
-      <c r="M22" s="90"/>
-      <c r="N22" s="90"/>
-      <c r="O22" s="91"/>
-      <c r="P22" s="64"/>
-    </row>
-    <row r="23" spans="1:16" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="114" t="s">
+      <c r="B23" s="124" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="116" t="s">
+      <c r="C23" s="125"/>
+      <c r="D23" s="128" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="117"/>
-      <c r="D23" s="120" t="s">
+      <c r="E23" s="129"/>
+      <c r="F23" s="124" t="s">
         <v>20</v>
       </c>
-      <c r="E23" s="121"/>
-      <c r="F23" s="116" t="s">
+      <c r="G23" s="125"/>
+      <c r="H23" s="124" t="s">
         <v>21</v>
       </c>
-      <c r="G23" s="117"/>
-      <c r="H23" s="116" t="s">
+      <c r="I23" s="125"/>
+      <c r="J23" s="124" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="117"/>
-      <c r="J23" s="116" t="s">
+      <c r="K23" s="125"/>
+      <c r="L23" s="132" t="s">
         <v>23</v>
       </c>
-      <c r="K23" s="117"/>
-      <c r="L23" s="124" t="s">
+      <c r="M23" s="133"/>
+      <c r="N23" s="136" t="s">
         <v>24</v>
       </c>
-      <c r="M23" s="125"/>
-      <c r="N23" s="128" t="s">
+      <c r="O23" s="136" t="s">
         <v>25</v>
       </c>
-      <c r="O23" s="128" t="s">
+      <c r="P23" s="64"/>
+    </row>
+    <row r="24" spans="1:16" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="123"/>
+      <c r="B24" s="126"/>
+      <c r="C24" s="127"/>
+      <c r="D24" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="P23" s="64"/>
-    </row>
-    <row r="24" spans="1:16" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="115"/>
-      <c r="B24" s="118"/>
-      <c r="C24" s="119"/>
-      <c r="D24" s="78" t="s">
+      <c r="E24" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="E24" s="78" t="s">
-        <v>28</v>
-      </c>
-      <c r="F24" s="122"/>
-      <c r="G24" s="123"/>
-      <c r="H24" s="118"/>
-      <c r="I24" s="119"/>
-      <c r="J24" s="122"/>
-      <c r="K24" s="123"/>
-      <c r="L24" s="126"/>
-      <c r="M24" s="127"/>
-      <c r="N24" s="129"/>
-      <c r="O24" s="129"/>
+      <c r="F24" s="130"/>
+      <c r="G24" s="131"/>
+      <c r="H24" s="126"/>
+      <c r="I24" s="127"/>
+      <c r="J24" s="130"/>
+      <c r="K24" s="131"/>
+      <c r="L24" s="134"/>
+      <c r="M24" s="135"/>
+      <c r="N24" s="137"/>
+      <c r="O24" s="137"/>
       <c r="P24" s="71" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:16" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="73">
         <v>1</v>
       </c>
-      <c r="B25" s="130"/>
-      <c r="C25" s="131"/>
+      <c r="B25" s="138"/>
+      <c r="C25" s="139"/>
       <c r="D25" s="16">
         <v>0</v>
       </c>
@@ -2154,11 +2151,11 @@
       <c r="P25" s="64"/>
     </row>
     <row r="26" spans="1:16" s="2" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="97" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" s="98"/>
-      <c r="C26" s="99"/>
+      <c r="A26" s="148" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="149"/>
+      <c r="C26" s="150"/>
       <c r="D26" s="25">
         <f>SUM(D25:D25)</f>
         <v>0</v>
@@ -2228,59 +2225,59 @@
       <c r="P27" s="60"/>
     </row>
     <row r="28" spans="1:16" s="2" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="93" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="96"/>
-      <c r="E28" s="96"/>
-      <c r="F28" s="94"/>
-      <c r="G28" s="94"/>
-      <c r="H28" s="94"/>
-      <c r="I28" s="94"/>
-      <c r="J28" s="94"/>
-      <c r="K28" s="94"/>
-      <c r="L28" s="94"/>
-      <c r="M28" s="94"/>
-      <c r="N28" s="94"/>
-      <c r="O28" s="95"/>
+      <c r="A28" s="91" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="92"/>
+      <c r="C28" s="92"/>
+      <c r="D28" s="93"/>
+      <c r="E28" s="93"/>
+      <c r="F28" s="92"/>
+      <c r="G28" s="92"/>
+      <c r="H28" s="92"/>
+      <c r="I28" s="92"/>
+      <c r="J28" s="92"/>
+      <c r="K28" s="92"/>
+      <c r="L28" s="92"/>
+      <c r="M28" s="92"/>
+      <c r="N28" s="92"/>
+      <c r="O28" s="94"/>
       <c r="P28" s="60"/>
     </row>
     <row r="29" spans="1:16" s="2" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="79" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B29" s="80" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" s="155" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="106" t="s">
+      <c r="D29" s="156"/>
+      <c r="E29" s="155" t="s">
+        <v>38</v>
+      </c>
+      <c r="F29" s="156"/>
+      <c r="G29" s="155" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="158"/>
-      <c r="E29" s="106" t="s">
-        <v>39</v>
-      </c>
-      <c r="F29" s="158"/>
-      <c r="G29" s="106" t="s">
+      <c r="H29" s="156"/>
+      <c r="I29" s="155" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="158"/>
-      <c r="I29" s="106" t="s">
+      <c r="J29" s="157"/>
+      <c r="K29" s="155" t="s">
         <v>43</v>
       </c>
-      <c r="J29" s="159"/>
-      <c r="K29" s="106" t="s">
+      <c r="L29" s="157"/>
+      <c r="M29" s="155" t="s">
         <v>44</v>
       </c>
-      <c r="L29" s="159"/>
-      <c r="M29" s="106" t="s">
-        <v>45</v>
-      </c>
-      <c r="N29" s="159"/>
-      <c r="O29" s="159"/>
+      <c r="N29" s="157"/>
+      <c r="O29" s="157"/>
       <c r="P29" s="72" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:16" s="2" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2290,55 +2287,55 @@
       <c r="B30" s="56"/>
       <c r="C30" s="75"/>
       <c r="D30" s="76"/>
-      <c r="E30" s="105"/>
-      <c r="F30" s="104"/>
+      <c r="E30" s="154"/>
+      <c r="F30" s="153"/>
       <c r="G30" s="77"/>
       <c r="H30" s="76"/>
-      <c r="I30" s="82"/>
-      <c r="J30" s="102"/>
-      <c r="K30" s="103"/>
-      <c r="L30" s="104"/>
-      <c r="M30" s="100"/>
-      <c r="N30" s="101"/>
-      <c r="O30" s="102"/>
+      <c r="I30" s="105"/>
+      <c r="J30" s="119"/>
+      <c r="K30" s="152"/>
+      <c r="L30" s="153"/>
+      <c r="M30" s="151"/>
+      <c r="N30" s="117"/>
+      <c r="O30" s="119"/>
       <c r="P30" s="63"/>
     </row>
     <row r="31" spans="1:16" s="2" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="149"/>
-      <c r="B31" s="150"/>
-      <c r="C31" s="151"/>
-      <c r="D31" s="149"/>
-      <c r="E31" s="152"/>
-      <c r="F31" s="153"/>
-      <c r="G31" s="154"/>
-      <c r="H31" s="149"/>
-      <c r="I31" s="155"/>
-      <c r="J31" s="151"/>
-      <c r="K31" s="152"/>
-      <c r="L31" s="153"/>
-      <c r="M31" s="151"/>
-      <c r="N31" s="151"/>
-      <c r="O31" s="151"/>
+      <c r="A31" s="82"/>
+      <c r="B31" s="83"/>
+      <c r="C31" s="84"/>
+      <c r="D31" s="82"/>
+      <c r="E31" s="85"/>
+      <c r="F31" s="86"/>
+      <c r="G31" s="87"/>
+      <c r="H31" s="82"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="84"/>
+      <c r="K31" s="85"/>
+      <c r="L31" s="86"/>
+      <c r="M31" s="84"/>
+      <c r="N31" s="84"/>
+      <c r="O31" s="84"/>
       <c r="P31" s="63"/>
     </row>
     <row r="32" spans="1:16" s="2" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="93"/>
-      <c r="B32" s="94"/>
-      <c r="C32" s="94"/>
-      <c r="D32" s="96"/>
-      <c r="E32" s="96"/>
-      <c r="F32" s="94"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="94"/>
-      <c r="I32" s="94"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="94"/>
-      <c r="L32" s="94"/>
-      <c r="M32" s="94"/>
-      <c r="N32" s="94"/>
-      <c r="O32" s="95"/>
+      <c r="A32" s="91"/>
+      <c r="B32" s="92"/>
+      <c r="C32" s="92"/>
+      <c r="D32" s="93"/>
+      <c r="E32" s="93"/>
+      <c r="F32" s="92"/>
+      <c r="G32" s="92"/>
+      <c r="H32" s="92"/>
+      <c r="I32" s="92"/>
+      <c r="J32" s="92"/>
+      <c r="K32" s="92"/>
+      <c r="L32" s="92"/>
+      <c r="M32" s="92"/>
+      <c r="N32" s="92"/>
+      <c r="O32" s="94"/>
       <c r="P32" s="63" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:16" s="2" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.25">
@@ -2352,27 +2349,27 @@
         <v>7</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F33" s="90" t="s">
+        <v>51</v>
+      </c>
+      <c r="G33" s="90"/>
+      <c r="H33" s="90"/>
+      <c r="I33" s="90"/>
+      <c r="J33" s="90" t="s">
         <v>52</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F33" s="139" t="s">
-        <v>53</v>
-      </c>
-      <c r="G33" s="139"/>
-      <c r="H33" s="139"/>
-      <c r="I33" s="139"/>
-      <c r="J33" s="139" t="s">
-        <v>54</v>
-      </c>
-      <c r="K33" s="139"/>
-      <c r="L33" s="139"/>
-      <c r="M33" s="139"/>
-      <c r="N33" s="139" t="s">
-        <v>45</v>
-      </c>
-      <c r="O33" s="139"/>
+      <c r="K33" s="90"/>
+      <c r="L33" s="90"/>
+      <c r="M33" s="90"/>
+      <c r="N33" s="90" t="s">
+        <v>44</v>
+      </c>
+      <c r="O33" s="90"/>
       <c r="P33" s="63"/>
     </row>
     <row r="34" spans="1:16" s="2" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2383,16 +2380,16 @@
       <c r="C34" s="42"/>
       <c r="D34" s="42"/>
       <c r="E34" s="42"/>
-      <c r="F34" s="156"/>
-      <c r="G34" s="156"/>
-      <c r="H34" s="156"/>
-      <c r="I34" s="156"/>
-      <c r="J34" s="157"/>
-      <c r="K34" s="157"/>
-      <c r="L34" s="157"/>
-      <c r="M34" s="157"/>
-      <c r="N34" s="157"/>
-      <c r="O34" s="157"/>
+      <c r="F34" s="88"/>
+      <c r="G34" s="88"/>
+      <c r="H34" s="88"/>
+      <c r="I34" s="88"/>
+      <c r="J34" s="89"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="89"/>
+      <c r="M34" s="89"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="89"/>
       <c r="P34" s="63"/>
     </row>
     <row r="35" spans="1:16" s="2" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2414,129 +2411,129 @@
       <c r="P35" s="60"/>
     </row>
     <row r="36" spans="1:16" s="2" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="93" t="s">
-        <v>31</v>
-      </c>
-      <c r="B36" s="94"/>
-      <c r="C36" s="94"/>
-      <c r="D36" s="94"/>
-      <c r="E36" s="94"/>
-      <c r="F36" s="94"/>
-      <c r="G36" s="94"/>
-      <c r="H36" s="94"/>
-      <c r="I36" s="94"/>
-      <c r="J36" s="94"/>
-      <c r="K36" s="94"/>
-      <c r="L36" s="94"/>
-      <c r="M36" s="94"/>
-      <c r="N36" s="94"/>
-      <c r="O36" s="95"/>
+      <c r="A36" s="91" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="92"/>
+      <c r="C36" s="92"/>
+      <c r="D36" s="92"/>
+      <c r="E36" s="92"/>
+      <c r="F36" s="92"/>
+      <c r="G36" s="92"/>
+      <c r="H36" s="92"/>
+      <c r="I36" s="92"/>
+      <c r="J36" s="92"/>
+      <c r="K36" s="92"/>
+      <c r="L36" s="92"/>
+      <c r="M36" s="92"/>
+      <c r="N36" s="92"/>
+      <c r="O36" s="94"/>
       <c r="P36" s="60"/>
     </row>
     <row r="37" spans="1:16" s="2" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="81" t="s">
-        <v>18</v>
-      </c>
-      <c r="B37" s="120" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="128" t="s">
+        <v>31</v>
+      </c>
+      <c r="C37" s="141"/>
+      <c r="D37" s="141"/>
+      <c r="E37" s="129"/>
+      <c r="F37" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="C37" s="133"/>
-      <c r="D37" s="133"/>
-      <c r="E37" s="121"/>
-      <c r="F37" s="120" t="s">
+      <c r="G37" s="141"/>
+      <c r="H37" s="141"/>
+      <c r="I37" s="141"/>
+      <c r="J37" s="141"/>
+      <c r="K37" s="141"/>
+      <c r="L37" s="129"/>
+      <c r="M37" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="G37" s="133"/>
-      <c r="H37" s="133"/>
-      <c r="I37" s="133"/>
-      <c r="J37" s="133"/>
-      <c r="K37" s="133"/>
-      <c r="L37" s="121"/>
-      <c r="M37" s="120" t="s">
-        <v>34</v>
-      </c>
-      <c r="N37" s="133"/>
-      <c r="O37" s="121"/>
+      <c r="N37" s="141"/>
+      <c r="O37" s="129"/>
       <c r="P37" s="60" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:16" s="2" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="56">
         <v>1</v>
       </c>
-      <c r="B38" s="82"/>
-      <c r="C38" s="92"/>
-      <c r="D38" s="92"/>
-      <c r="E38" s="107"/>
-      <c r="F38" s="82"/>
-      <c r="G38" s="92"/>
-      <c r="H38" s="92"/>
-      <c r="I38" s="92"/>
-      <c r="J38" s="92"/>
-      <c r="K38" s="92"/>
-      <c r="L38" s="107"/>
-      <c r="M38" s="108"/>
-      <c r="N38" s="109"/>
-      <c r="O38" s="110"/>
+      <c r="B38" s="105"/>
+      <c r="C38" s="142"/>
+      <c r="D38" s="142"/>
+      <c r="E38" s="143"/>
+      <c r="F38" s="105"/>
+      <c r="G38" s="142"/>
+      <c r="H38" s="142"/>
+      <c r="I38" s="142"/>
+      <c r="J38" s="142"/>
+      <c r="K38" s="142"/>
+      <c r="L38" s="143"/>
+      <c r="M38" s="144"/>
+      <c r="N38" s="145"/>
+      <c r="O38" s="146"/>
       <c r="P38" s="60"/>
     </row>
     <row r="39" spans="1:16" s="2" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="53"/>
       <c r="B39" s="53"/>
-      <c r="C39" s="111" t="s">
-        <v>51</v>
-      </c>
-      <c r="D39" s="111"/>
-      <c r="E39" s="111"/>
-      <c r="F39" s="111"/>
-      <c r="G39" s="111"/>
+      <c r="C39" s="147" t="s">
+        <v>50</v>
+      </c>
+      <c r="D39" s="147"/>
+      <c r="E39" s="147"/>
+      <c r="F39" s="147"/>
+      <c r="G39" s="147"/>
       <c r="H39" s="53"/>
       <c r="I39" s="53"/>
       <c r="J39" s="53"/>
       <c r="K39" s="53"/>
-      <c r="L39" s="111" t="s">
-        <v>49</v>
-      </c>
-      <c r="M39" s="111"/>
-      <c r="N39" s="111"/>
+      <c r="L39" s="147" t="s">
+        <v>48</v>
+      </c>
+      <c r="M39" s="147"/>
+      <c r="N39" s="147"/>
       <c r="O39" s="53"/>
       <c r="P39" s="59"/>
     </row>
     <row r="40" spans="1:16" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A40" s="132"/>
-      <c r="B40" s="132"/>
-      <c r="C40" s="132"/>
-      <c r="D40" s="132"/>
-      <c r="E40" s="132"/>
-      <c r="F40" s="132"/>
-      <c r="G40" s="132"/>
-      <c r="H40" s="132"/>
-      <c r="I40" s="132"/>
-      <c r="J40" s="132"/>
-      <c r="K40" s="132"/>
-      <c r="L40" s="132"/>
-      <c r="M40" s="132"/>
-      <c r="N40" s="132"/>
-      <c r="O40" s="132"/>
+      <c r="A40" s="140"/>
+      <c r="B40" s="140"/>
+      <c r="C40" s="140"/>
+      <c r="D40" s="140"/>
+      <c r="E40" s="140"/>
+      <c r="F40" s="140"/>
+      <c r="G40" s="140"/>
+      <c r="H40" s="140"/>
+      <c r="I40" s="140"/>
+      <c r="J40" s="140"/>
+      <c r="K40" s="140"/>
+      <c r="L40" s="140"/>
+      <c r="M40" s="140"/>
+      <c r="N40" s="140"/>
+      <c r="O40" s="140"/>
       <c r="P40" s="59"/>
     </row>
     <row r="41" spans="1:16" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A41" s="132"/>
-      <c r="B41" s="132"/>
-      <c r="C41" s="132"/>
-      <c r="D41" s="132"/>
-      <c r="E41" s="132"/>
-      <c r="F41" s="132"/>
-      <c r="G41" s="132"/>
-      <c r="H41" s="132"/>
-      <c r="I41" s="132"/>
-      <c r="J41" s="132"/>
-      <c r="K41" s="132"/>
-      <c r="L41" s="132"/>
-      <c r="M41" s="132"/>
-      <c r="N41" s="132"/>
-      <c r="O41" s="132"/>
+      <c r="A41" s="140"/>
+      <c r="B41" s="140"/>
+      <c r="C41" s="140"/>
+      <c r="D41" s="140"/>
+      <c r="E41" s="140"/>
+      <c r="F41" s="140"/>
+      <c r="G41" s="140"/>
+      <c r="H41" s="140"/>
+      <c r="I41" s="140"/>
+      <c r="J41" s="140"/>
+      <c r="K41" s="140"/>
+      <c r="L41" s="140"/>
+      <c r="M41" s="140"/>
+      <c r="N41" s="140"/>
+      <c r="O41" s="140"/>
       <c r="P41" s="59"/>
     </row>
     <row r="42" spans="1:16" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
@@ -2901,13 +2898,13 @@
     </row>
     <row r="107" spans="17:26" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="108" spans="17:26" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="R108" s="112"/>
-      <c r="S108" s="112"/>
-      <c r="T108" s="112"/>
-      <c r="V108" s="112"/>
-      <c r="W108" s="112"/>
-      <c r="X108" s="112"/>
-      <c r="Z108" s="113"/>
+      <c r="R108" s="120"/>
+      <c r="S108" s="120"/>
+      <c r="T108" s="120"/>
+      <c r="V108" s="120"/>
+      <c r="W108" s="120"/>
+      <c r="X108" s="120"/>
+      <c r="Z108" s="121"/>
     </row>
     <row r="109" spans="17:26" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="R109" s="66"/>
@@ -2916,7 +2913,7 @@
       <c r="V109" s="66"/>
       <c r="W109" s="66"/>
       <c r="X109" s="66"/>
-      <c r="Z109" s="113"/>
+      <c r="Z109" s="121"/>
     </row>
     <row r="110" spans="17:26" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="R110" s="66"/>
@@ -3183,32 +3180,32 @@
     <row r="201" spans="17:18" ht="37.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="68">
-    <mergeCell ref="F34:I34"/>
-    <mergeCell ref="J34:M34"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="J33:M33"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="A32:O32"/>
-    <mergeCell ref="A22:O22"/>
-    <mergeCell ref="A21:O21"/>
-    <mergeCell ref="E15:M15"/>
-    <mergeCell ref="A17:O17"/>
-    <mergeCell ref="E19:M19"/>
-    <mergeCell ref="E20:M20"/>
-    <mergeCell ref="E18:I18"/>
-    <mergeCell ref="E9:I9"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A3:O3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="F4:O4"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="F6:O6"/>
-    <mergeCell ref="A7:O7"/>
-    <mergeCell ref="A8:O8"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="F5:O5"/>
+    <mergeCell ref="E10:I10"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="E14:I14"/>
+    <mergeCell ref="E11:M11"/>
+    <mergeCell ref="A12:O12"/>
+    <mergeCell ref="A13:O13"/>
+    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="A36:O36"/>
+    <mergeCell ref="A28:O28"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="M30:O30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="M29:O29"/>
+    <mergeCell ref="M37:O37"/>
+    <mergeCell ref="F38:L38"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="M38:O38"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="L39:N39"/>
     <mergeCell ref="V108:X108"/>
     <mergeCell ref="Z108:Z109"/>
     <mergeCell ref="A23:A24"/>
@@ -3225,32 +3222,32 @@
     <mergeCell ref="A40:O41"/>
     <mergeCell ref="B37:E37"/>
     <mergeCell ref="F37:L37"/>
-    <mergeCell ref="M37:O37"/>
-    <mergeCell ref="F38:L38"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="M38:O38"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="L39:N39"/>
-    <mergeCell ref="A36:O36"/>
-    <mergeCell ref="A28:O28"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="M30:O30"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="M29:O29"/>
-    <mergeCell ref="E10:I10"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="E14:I14"/>
-    <mergeCell ref="E11:M11"/>
-    <mergeCell ref="A12:O12"/>
-    <mergeCell ref="A13:O13"/>
-    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="E9:I9"/>
+    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="F4:O4"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="F6:O6"/>
+    <mergeCell ref="A7:O7"/>
+    <mergeCell ref="A8:O8"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="F5:O5"/>
+    <mergeCell ref="A32:O32"/>
+    <mergeCell ref="A22:O22"/>
+    <mergeCell ref="A21:O21"/>
+    <mergeCell ref="E15:M15"/>
+    <mergeCell ref="A17:O17"/>
+    <mergeCell ref="E19:M19"/>
+    <mergeCell ref="E20:M20"/>
+    <mergeCell ref="E18:I18"/>
+    <mergeCell ref="F34:I34"/>
+    <mergeCell ref="J34:M34"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="J33:M33"/>
+    <mergeCell ref="N33:O33"/>
   </mergeCells>
   <phoneticPr fontId="24" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>